<commit_message>
Accomplished upto 14 testcases
</commit_message>
<xml_diff>
--- a/src/test/resources/Files/TestData.XLSX
+++ b/src/test/resources/Files/TestData.XLSX
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GHEMobileAutomation\GHEMobileAutomation\src\test\resources\Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1120AF78-C73B-4663-8611-CE7FE7E263B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFD538B4-8611-4BD7-9BCA-A66430604479}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginPage" sheetId="17" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="233">
   <si>
     <t>Key</t>
   </si>
@@ -698,6 +698,45 @@
   </si>
   <si>
     <t>Thank you for your question/comments. We will get back to you as soon as possible.</t>
+  </si>
+  <si>
+    <t>MessageToBeReply</t>
+  </si>
+  <si>
+    <t>This message is replied manually for checking purpose</t>
+  </si>
+  <si>
+    <t>https://v2.tailwindcss.com/docs</t>
+  </si>
+  <si>
+    <t>MessageToBeReplyAsHyperLink</t>
+  </si>
+  <si>
+    <t>InvalidUserNameForHW</t>
+  </si>
+  <si>
+    <t>qm111@test.com</t>
+  </si>
+  <si>
+    <t>InvalidPasswordForHW</t>
+  </si>
+  <si>
+    <t>Abcd123</t>
+  </si>
+  <si>
+    <t>LoginErrorMessage</t>
+  </si>
+  <si>
+    <t>ExpectedHeaderForEmptyMessagesInInbox</t>
+  </si>
+  <si>
+    <t>ExpectedTextForEmptyMessagesInInbox</t>
+  </si>
+  <si>
+    <t>ErrorTextForInvalidUserName</t>
+  </si>
+  <si>
+    <t>ErrorTextForInvalidPassword</t>
   </si>
 </sst>
 </file>
@@ -746,7 +785,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -767,6 +806,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -983,7 +1023,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="38.69921875" style="1" bestFit="1" customWidth="1"/>
@@ -1199,18 +1239,59 @@
         <v>213</v>
       </c>
     </row>
+    <row r="27" spans="1:2">
+      <c r="A27" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2">
+      <c r="A28" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2">
+      <c r="A29" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2">
+      <c r="A30" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2">
+      <c r="A31" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" xr:uid="{F19F960E-407D-4B4E-AECF-B1E4E88A0143}"/>
+    <hyperlink ref="B27" r:id="rId2" xr:uid="{CA7700A4-865E-4033-ADC6-D924301F4506}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId2"/>
+  <pageSetup orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B779F2E-73BC-41B4-9D32-F94A736A4465}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="44.69921875" customWidth="1"/>
@@ -1249,7 +1330,42 @@
         <v>219</v>
       </c>
     </row>
+    <row r="5" spans="1:2">
+      <c r="A5" t="s">
+        <v>220</v>
+      </c>
+      <c r="B5" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" t="s">
+        <v>223</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" t="s">
+        <v>229</v>
+      </c>
+      <c r="B7" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" t="s">
+        <v>230</v>
+      </c>
+      <c r="B8" t="s">
+        <v>127</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B6" r:id="rId1" xr:uid="{B37CC70B-4934-4F54-9557-5E1382F818CC}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Completed and executed 23 testcases successfully and updated the readme file with some xml files
</commit_message>
<xml_diff>
--- a/src/test/resources/Files/TestData.XLSX
+++ b/src/test/resources/Files/TestData.XLSX
@@ -8,17 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GHEMobileAutomation\GHEMobileAutomation\src\test\resources\Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFD538B4-8611-4BD7-9BCA-A66430604479}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CDDFBAD-FC93-4423-9AA1-D9F45CCC443F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginPage" sheetId="17" r:id="rId1"/>
-    <sheet name="InboxPage" sheetId="22" r:id="rId2"/>
-    <sheet name="HomePage" sheetId="18" r:id="rId3"/>
-    <sheet name="DocumentPage" sheetId="19" r:id="rId4"/>
-    <sheet name="MessagePage" sheetId="20" r:id="rId5"/>
-    <sheet name="UploadPage" sheetId="21" r:id="rId6"/>
+    <sheet name="SurveysPage" sheetId="23" r:id="rId2"/>
+    <sheet name="InboxPage" sheetId="22" r:id="rId3"/>
+    <sheet name="HomePage" sheetId="18" r:id="rId4"/>
+    <sheet name="DocumentPage" sheetId="19" r:id="rId5"/>
+    <sheet name="MessagePage" sheetId="20" r:id="rId6"/>
+    <sheet name="UploadPage" sheetId="21" r:id="rId7"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="254">
   <si>
     <t>Key</t>
   </si>
@@ -737,6 +738,69 @@
   </si>
   <si>
     <t>ErrorTextForInvalidPassword</t>
+  </si>
+  <si>
+    <t>UserNameNoActiveSurvey</t>
+  </si>
+  <si>
+    <t>UserNameNoCompletedSurvey</t>
+  </si>
+  <si>
+    <t>qm1004@test.com</t>
+  </si>
+  <si>
+    <t>SurveyCenterTitle</t>
+  </si>
+  <si>
+    <t>Survey Center</t>
+  </si>
+  <si>
+    <t>SurveyCenterWelcomeMessage</t>
+  </si>
+  <si>
+    <t>Welcome to the Survey Center</t>
+  </si>
+  <si>
+    <t>SurveyCenterWelcomeText</t>
+  </si>
+  <si>
+    <t>Click on any of the Active surveys to provide your answers before the expiration date. Each survey should take about 5 minutes to complete. Most of the surveys help your Coach understand your current thoughts and feelings about your health and weight loss journey.</t>
+  </si>
+  <si>
+    <t>NoSurveysMessage</t>
+  </si>
+  <si>
+    <t>No surveys found</t>
+  </si>
+  <si>
+    <t>NoSurveysText</t>
+  </si>
+  <si>
+    <t>You do not have any surveys currently.</t>
+  </si>
+  <si>
+    <t>CompletedSurveysScreenTitle</t>
+  </si>
+  <si>
+    <t>Completed Surveys</t>
+  </si>
+  <si>
+    <t>ActiveSurveysScreenTitle</t>
+  </si>
+  <si>
+    <t>Active Surveys</t>
+  </si>
+  <si>
+    <t>UserNameForInboxMessageValidation</t>
+  </si>
+  <si>
+    <t>qm1022@test.com</t>
+  </si>
+  <si>
+    <t>UserNameForInboxMessagesCount</t>
+  </si>
+  <si>
+    <t>qm1021@test.com</t>
   </si>
 </sst>
 </file>
@@ -1023,7 +1087,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
-  <dimension ref="A1:B31"/>
+  <dimension ref="A1:B35"/>
   <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="38.69921875" style="1" bestFit="1" customWidth="1"/>
@@ -1279,17 +1343,131 @@
         <v>6</v>
       </c>
     </row>
+    <row r="32" spans="1:2">
+      <c r="A32" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2">
+      <c r="A33" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2">
+      <c r="A34" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2">
+      <c r="A35" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>253</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" xr:uid="{F19F960E-407D-4B4E-AECF-B1E4E88A0143}"/>
     <hyperlink ref="B27" r:id="rId2" xr:uid="{CA7700A4-865E-4033-ADC6-D924301F4506}"/>
+    <hyperlink ref="B32" r:id="rId3" xr:uid="{68EDD19A-2DC2-4930-925B-CF86A1F7842B}"/>
+    <hyperlink ref="B33" r:id="rId4" xr:uid="{C05F0A0E-BCD2-4430-89C0-994A4AE4CA92}"/>
+    <hyperlink ref="B34" r:id="rId5" xr:uid="{6F80331E-EDF8-4B25-BB4C-5D621976AD84}"/>
+    <hyperlink ref="B35" r:id="rId6" xr:uid="{7440F14C-4607-4D53-B467-7038D2ECB3B2}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId3"/>
+  <pageSetup orientation="portrait" r:id="rId7"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A0B0156-F803-4942-AB8F-C1FD93E603F0}">
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
+  <cols>
+    <col min="1" max="1" width="27.8984375" customWidth="1"/>
+    <col min="2" max="2" width="57.69921875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="55.2">
+      <c r="A4" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>249</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B779F2E-73BC-41B4-9D32-F94A736A4465}">
   <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
@@ -1370,7 +1548,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52DF3179-8EA4-4C07-A99A-335D7C63B22A}">
   <dimension ref="A1:B62"/>
   <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="13.8"/>
@@ -1884,7 +2062,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37394D8A-5B1E-4B1E-AA1A-5AC45A93E45C}">
   <dimension ref="A1:O12"/>
   <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="13.8"/>
@@ -1997,7 +2175,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D79144E4-9B96-4467-B95A-F62A7D36273F}">
   <dimension ref="A1:B5"/>
   <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="13.8"/>
@@ -2048,7 +2226,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54745E9E-4F33-4295-B25E-6A99C03B8E97}">
   <dimension ref="A1:B8"/>
   <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="13.8"/>

</xml_diff>